<commit_message>
Update daily ventilation data
</commit_message>
<xml_diff>
--- a/data/ventilation.xlsx
+++ b/data/ventilation.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.348156+07:00</t>
+          <t>2026-10-30T09:57:41.150174+07:00</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.878367+07:00</t>
+          <t>2026-10-30T09:57:08.214173+07:00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.898034+07:00</t>
+          <t>2026-10-30T09:57:34.038244+07:00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.507936+07:00</t>
+          <t>2026-10-30T09:57:23.444750+07:00</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.149270+07:00</t>
+          <t>2026-10-30T09:57:18.069775+07:00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:38.320126+07:00</t>
+          <t>2026-10-30T09:57:19.864257+07:00</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:57.120352+07:00</t>
+          <t>2026-10-30T09:57:35.895575+07:00</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.898961+07:00</t>
+          <t>2026-10-30T09:57:34.105301+07:00</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.902569+07:00</t>
+          <t>2026-10-30T09:57:34.105945+07:00</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:49.026297+07:00</t>
+          <t>2026-10-30T09:57:28.764491+07:00</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.636144+07:00</t>
+          <t>2026-10-30T09:57:25.222675+07:00</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.470505+07:00</t>
+          <t>2026-10-30T09:57:39.341789+07:00</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.577304+07:00</t>
+          <t>2026-10-30T09:57:42.697769+07:00</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.626476+07:00</t>
+          <t>2026-10-30T09:57:37.519884+07:00</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.789485+07:00</t>
+          <t>2026-10-30T09:57:15.520662+07:00</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.952321+07:00</t>
+          <t>2026-10-30T09:57:30.544292+07:00</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.844881+07:00</t>
+          <t>2026-10-30T09:57:10.943146+07:00</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.189007+07:00</t>
+          <t>2026-10-30T09:57:21.654228+07:00</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:47.325100+07:00</t>
+          <t>2026-10-30T09:57:27.002543+07:00</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.292980+07:00</t>
+          <t>2026-10-30T09:57:41.134961+07:00</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.658010+07:00</t>
+          <t>2026-10-30T09:57:28.724576+07:00</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879040+07:00</t>
+          <t>2026-10-30T09:57:08.214851+07:00</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:06.382959+07:00</t>
+          <t>2026-10-30T09:57:44.377183+07:00</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.954128+07:00</t>
+          <t>2026-10-30T09:57:13.590283+07:00</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:38.321311+07:00</t>
+          <t>2026-10-30T09:57:19.882864+07:00</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.430381+07:00</t>
+          <t>2026-10-30T09:57:26.959820+07:00</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879433+07:00</t>
+          <t>2026-10-30T09:57:08.215245+07:00</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.407963+07:00</t>
+          <t>2026-10-30T09:57:39.268142+07:00</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.663643+07:00</t>
+          <t>2026-10-30T09:57:35.813589+07:00</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.578390+07:00</t>
+          <t>2026-10-30T09:57:42.901581+07:00</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.950800+07:00</t>
+          <t>2026-10-30T09:57:30.513158+07:00</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.916754+07:00</t>
+          <t>2026-10-30T09:57:13.587818+07:00</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.219072+07:00</t>
+          <t>2026-10-30T09:57:40.995154+07:00</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.460235+07:00</t>
+          <t>2026-10-30T09:57:41.168176+07:00</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.151040+07:00</t>
+          <t>2026-10-30T09:57:18.104399+07:00</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.136269+07:00</t>
+          <t>2026-10-30T09:57:18.063447+07:00</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.708619+07:00</t>
+          <t>2026-10-30T09:57:37.640408+07:00</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.613919+07:00</t>
+          <t>2026-10-30T09:57:25.150379+07:00</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.506876+07:00</t>
+          <t>2026-10-30T09:57:23.403713+07:00</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.615429+07:00</t>
+          <t>2026-10-30T09:57:42.920119+07:00</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.317606+07:00</t>
+          <t>2026-10-30T09:57:26.958822+07:00</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.546220+07:00</t>
+          <t>2026-10-30T09:57:39.399308+07:00</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.614764+07:00</t>
+          <t>2026-10-30T09:57:35.774483+07:00</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.041835+07:00</t>
+          <t>2026-10-30T09:57:32.267505+07:00</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.614845+07:00</t>
+          <t>2026-10-30T09:57:25.187837+07:00</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.043505+07:00</t>
+          <t>2026-10-30T09:57:32.338309+07:00</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.788158+07:00</t>
+          <t>2026-10-30T09:57:15.230449+07:00</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.954863+07:00</t>
+          <t>2026-10-30T09:57:13.605705+07:00</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.431445+07:00</t>
+          <t>2026-10-30T09:57:26.960653+07:00</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.493622+07:00</t>
+          <t>2026-10-30T09:57:23.402806+07:00</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.687237+07:00</t>
+          <t>2026-10-30T09:57:37.572573+07:00</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.579683+07:00</t>
+          <t>2026-10-30T09:57:42.919200+07:00</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879945+07:00</t>
+          <t>2026-10-30T09:57:08.215829+07:00</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.894727+07:00</t>
+          <t>2026-10-30T09:57:34.006892+07:00</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.845442+07:00</t>
+          <t>2026-10-30T09:57:10.943711+07:00</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.041011+07:00</t>
+          <t>2026-10-30T09:57:32.265183+07:00</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.702074+07:00</t>
+          <t>2026-10-30T09:57:35.857622+07:00</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.951722+07:00</t>
+          <t>2026-10-30T09:57:30.533140+07:00</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.042937+07:00</t>
+          <t>2026-10-30T09:57:32.317455+07:00</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.671439+07:00</t>
+          <t>2026-10-30T09:57:39.416999+07:00</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.594388+07:00</t>
+          <t>2026-10-30T09:57:28.723532+07:00</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.135506+07:00</t>
+          <t>2026-10-30T09:57:18.062473+07:00</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.148730+07:00</t>
+          <t>2026-10-30T09:57:21.606230+07:00</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.492614+07:00</t>
+          <t>2026-10-30T09:57:23.362870+07:00</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.615639+07:00</t>
+          <t>2026-10-30T09:57:25.199315+07:00</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.191795+07:00</t>
+          <t>2026-10-30T09:57:21.654901+07:00</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.790040+07:00</t>
+          <t>2026-10-30T09:57:15.526309+07:00</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.689393+07:00</t>
+          <t>2026-10-30T09:57:28.754114+07:00</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:37.816883+07:00</t>
+          <t>2026-10-30T09:57:19.840148+07:00</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.949592+07:00</t>
+          <t>2026-10-30T09:57:30.484548+07:00</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.847007+07:00</t>
+          <t>2026-10-30T09:57:10.944880+07:00</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.846368+07:00</t>
+          <t>2026-10-30T09:57:10.944223+07:00</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.905897+07:00</t>
+          <t>2026-10-30T09:57:37.665275+07:00</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:37.816068+07:00</t>
+          <t>2026-10-30T09:57:19.827952+07:00</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.150024+07:00</t>
+          <t>2026-10-30T09:57:21.607153+07:00</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.788912+07:00</t>
+          <t>2026-10-30T09:57:15.300415+07:00</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.915990+07:00</t>
+          <t>2026-10-30T09:57:13.561604+07:00</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -35283,7 +35283,7 @@
       </c>
       <c r="G772" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.348156+07:00</t>
+          <t>2026-10-30T09:57:41.150174+07:00</t>
         </is>
       </c>
       <c r="H772" s="2" t="inlineStr">
@@ -35324,7 +35324,7 @@
       </c>
       <c r="G773" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.878367+07:00</t>
+          <t>2026-10-30T09:57:08.214173+07:00</t>
         </is>
       </c>
       <c r="H773" s="2" t="inlineStr">
@@ -35365,7 +35365,7 @@
       </c>
       <c r="G774" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.898034+07:00</t>
+          <t>2026-10-30T09:57:34.038244+07:00</t>
         </is>
       </c>
       <c r="H774" s="2" t="inlineStr">
@@ -35406,7 +35406,7 @@
       </c>
       <c r="G775" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.507936+07:00</t>
+          <t>2026-10-30T09:57:23.444750+07:00</t>
         </is>
       </c>
       <c r="H775" s="2" t="inlineStr">
@@ -35447,7 +35447,7 @@
       </c>
       <c r="G776" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.149270+07:00</t>
+          <t>2026-10-30T09:57:18.069775+07:00</t>
         </is>
       </c>
       <c r="H776" s="2" t="inlineStr">
@@ -35488,7 +35488,7 @@
       </c>
       <c r="G777" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:38.320126+07:00</t>
+          <t>2026-10-30T09:57:19.864257+07:00</t>
         </is>
       </c>
       <c r="H777" s="2" t="inlineStr">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="G778" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:57.120352+07:00</t>
+          <t>2026-10-30T09:57:35.895575+07:00</t>
         </is>
       </c>
       <c r="H778" s="2" t="inlineStr">
@@ -35570,7 +35570,7 @@
       </c>
       <c r="G779" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.898961+07:00</t>
+          <t>2026-10-30T09:57:34.105301+07:00</t>
         </is>
       </c>
       <c r="H779" s="2" t="inlineStr">
@@ -35611,7 +35611,7 @@
       </c>
       <c r="G780" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.902569+07:00</t>
+          <t>2026-10-30T09:57:34.105945+07:00</t>
         </is>
       </c>
       <c r="H780" s="2" t="inlineStr">
@@ -35652,7 +35652,7 @@
       </c>
       <c r="G781" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:49.026297+07:00</t>
+          <t>2026-10-30T09:57:28.764491+07:00</t>
         </is>
       </c>
       <c r="H781" s="2" t="inlineStr">
@@ -35693,7 +35693,7 @@
       </c>
       <c r="G782" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.636144+07:00</t>
+          <t>2026-10-30T09:57:25.222675+07:00</t>
         </is>
       </c>
       <c r="H782" s="2" t="inlineStr">
@@ -35734,7 +35734,7 @@
       </c>
       <c r="G783" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.470505+07:00</t>
+          <t>2026-10-30T09:57:39.341789+07:00</t>
         </is>
       </c>
       <c r="H783" s="2" t="inlineStr">
@@ -35775,7 +35775,7 @@
       </c>
       <c r="G784" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.577304+07:00</t>
+          <t>2026-10-30T09:57:42.697769+07:00</t>
         </is>
       </c>
       <c r="H784" s="2" t="inlineStr">
@@ -35816,7 +35816,7 @@
       </c>
       <c r="G785" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.626476+07:00</t>
+          <t>2026-10-30T09:57:37.519884+07:00</t>
         </is>
       </c>
       <c r="H785" s="2" t="inlineStr">
@@ -35857,7 +35857,7 @@
       </c>
       <c r="G786" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.789485+07:00</t>
+          <t>2026-10-30T09:57:15.520662+07:00</t>
         </is>
       </c>
       <c r="H786" s="2" t="inlineStr">
@@ -35898,7 +35898,7 @@
       </c>
       <c r="G787" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.952321+07:00</t>
+          <t>2026-10-30T09:57:30.544292+07:00</t>
         </is>
       </c>
       <c r="H787" s="2" t="inlineStr">
@@ -35939,7 +35939,7 @@
       </c>
       <c r="G788" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.844881+07:00</t>
+          <t>2026-10-30T09:57:10.943146+07:00</t>
         </is>
       </c>
       <c r="H788" s="2" t="inlineStr">
@@ -35980,7 +35980,7 @@
       </c>
       <c r="G789" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.189007+07:00</t>
+          <t>2026-10-30T09:57:21.654228+07:00</t>
         </is>
       </c>
       <c r="H789" s="2" t="inlineStr">
@@ -36021,7 +36021,7 @@
       </c>
       <c r="G790" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:47.325100+07:00</t>
+          <t>2026-10-30T09:57:27.002543+07:00</t>
         </is>
       </c>
       <c r="H790" s="2" t="inlineStr">
@@ -36062,7 +36062,7 @@
       </c>
       <c r="G791" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.292980+07:00</t>
+          <t>2026-10-30T09:57:41.134961+07:00</t>
         </is>
       </c>
       <c r="H791" s="2" t="inlineStr">
@@ -36103,7 +36103,7 @@
       </c>
       <c r="G792" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.658010+07:00</t>
+          <t>2026-10-30T09:57:28.724576+07:00</t>
         </is>
       </c>
       <c r="H792" s="2" t="inlineStr">
@@ -36144,7 +36144,7 @@
       </c>
       <c r="G793" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879040+07:00</t>
+          <t>2026-10-30T09:57:08.214851+07:00</t>
         </is>
       </c>
       <c r="H793" s="2" t="inlineStr">
@@ -36185,7 +36185,7 @@
       </c>
       <c r="G794" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:06.382959+07:00</t>
+          <t>2026-10-30T09:57:44.377183+07:00</t>
         </is>
       </c>
       <c r="H794" s="2" t="inlineStr">
@@ -36226,7 +36226,7 @@
       </c>
       <c r="G795" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.954128+07:00</t>
+          <t>2026-10-30T09:57:13.590283+07:00</t>
         </is>
       </c>
       <c r="H795" s="2" t="inlineStr">
@@ -36267,7 +36267,7 @@
       </c>
       <c r="G796" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:38.321311+07:00</t>
+          <t>2026-10-30T09:57:19.882864+07:00</t>
         </is>
       </c>
       <c r="H796" s="2" t="inlineStr">
@@ -36308,7 +36308,7 @@
       </c>
       <c r="G797" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.430381+07:00</t>
+          <t>2026-10-30T09:57:26.959820+07:00</t>
         </is>
       </c>
       <c r="H797" s="2" t="inlineStr">
@@ -36349,7 +36349,7 @@
       </c>
       <c r="G798" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879433+07:00</t>
+          <t>2026-10-30T09:57:08.215245+07:00</t>
         </is>
       </c>
       <c r="H798" s="2" t="inlineStr">
@@ -36390,7 +36390,7 @@
       </c>
       <c r="G799" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.407963+07:00</t>
+          <t>2026-10-30T09:57:39.268142+07:00</t>
         </is>
       </c>
       <c r="H799" s="2" t="inlineStr">
@@ -36431,7 +36431,7 @@
       </c>
       <c r="G800" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.663643+07:00</t>
+          <t>2026-10-30T09:57:35.813589+07:00</t>
         </is>
       </c>
       <c r="H800" s="2" t="inlineStr">
@@ -36472,7 +36472,7 @@
       </c>
       <c r="G801" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.578390+07:00</t>
+          <t>2026-10-30T09:57:42.901581+07:00</t>
         </is>
       </c>
       <c r="H801" s="2" t="inlineStr">
@@ -36513,7 +36513,7 @@
       </c>
       <c r="G802" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.950800+07:00</t>
+          <t>2026-10-30T09:57:30.513158+07:00</t>
         </is>
       </c>
       <c r="H802" s="2" t="inlineStr">
@@ -36554,7 +36554,7 @@
       </c>
       <c r="G803" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.916754+07:00</t>
+          <t>2026-10-30T09:57:13.587818+07:00</t>
         </is>
       </c>
       <c r="H803" s="2" t="inlineStr">
@@ -36595,7 +36595,7 @@
       </c>
       <c r="G804" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.219072+07:00</t>
+          <t>2026-10-30T09:57:40.995154+07:00</t>
         </is>
       </c>
       <c r="H804" s="2" t="inlineStr">
@@ -36636,7 +36636,7 @@
       </c>
       <c r="G805" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:02.460235+07:00</t>
+          <t>2026-10-30T09:57:41.168176+07:00</t>
         </is>
       </c>
       <c r="H805" s="2" t="inlineStr">
@@ -36677,7 +36677,7 @@
       </c>
       <c r="G806" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.151040+07:00</t>
+          <t>2026-10-30T09:57:18.104399+07:00</t>
         </is>
       </c>
       <c r="H806" s="2" t="inlineStr">
@@ -36718,7 +36718,7 @@
       </c>
       <c r="G807" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.136269+07:00</t>
+          <t>2026-10-30T09:57:18.063447+07:00</t>
         </is>
       </c>
       <c r="H807" s="2" t="inlineStr">
@@ -36759,7 +36759,7 @@
       </c>
       <c r="G808" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.708619+07:00</t>
+          <t>2026-10-30T09:57:37.640408+07:00</t>
         </is>
       </c>
       <c r="H808" s="2" t="inlineStr">
@@ -36800,7 +36800,7 @@
       </c>
       <c r="G809" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.613919+07:00</t>
+          <t>2026-10-30T09:57:25.150379+07:00</t>
         </is>
       </c>
       <c r="H809" s="2" t="inlineStr">
@@ -36841,7 +36841,7 @@
       </c>
       <c r="G810" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.506876+07:00</t>
+          <t>2026-10-30T09:57:23.403713+07:00</t>
         </is>
       </c>
       <c r="H810" s="2" t="inlineStr">
@@ -36882,7 +36882,7 @@
       </c>
       <c r="G811" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.615429+07:00</t>
+          <t>2026-10-30T09:57:42.920119+07:00</t>
         </is>
       </c>
       <c r="H811" s="2" t="inlineStr">
@@ -36923,7 +36923,7 @@
       </c>
       <c r="G812" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.317606+07:00</t>
+          <t>2026-10-30T09:57:26.958822+07:00</t>
         </is>
       </c>
       <c r="H812" s="2" t="inlineStr">
@@ -36964,7 +36964,7 @@
       </c>
       <c r="G813" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.546220+07:00</t>
+          <t>2026-10-30T09:57:39.399308+07:00</t>
         </is>
       </c>
       <c r="H813" s="2" t="inlineStr">
@@ -37005,7 +37005,7 @@
       </c>
       <c r="G814" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.614764+07:00</t>
+          <t>2026-10-30T09:57:35.774483+07:00</t>
         </is>
       </c>
       <c r="H814" s="2" t="inlineStr">
@@ -37046,7 +37046,7 @@
       </c>
       <c r="G815" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.041835+07:00</t>
+          <t>2026-10-30T09:57:32.267505+07:00</t>
         </is>
       </c>
       <c r="H815" s="2" t="inlineStr">
@@ -37087,7 +37087,7 @@
       </c>
       <c r="G816" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.614845+07:00</t>
+          <t>2026-10-30T09:57:25.187837+07:00</t>
         </is>
       </c>
       <c r="H816" s="2" t="inlineStr">
@@ -37128,7 +37128,7 @@
       </c>
       <c r="G817" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.043505+07:00</t>
+          <t>2026-10-30T09:57:32.338309+07:00</t>
         </is>
       </c>
       <c r="H817" s="2" t="inlineStr">
@@ -37169,7 +37169,7 @@
       </c>
       <c r="G818" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.788158+07:00</t>
+          <t>2026-10-30T09:57:15.230449+07:00</t>
         </is>
       </c>
       <c r="H818" s="2" t="inlineStr">
@@ -37210,7 +37210,7 @@
       </c>
       <c r="G819" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.954863+07:00</t>
+          <t>2026-10-30T09:57:13.605705+07:00</t>
         </is>
       </c>
       <c r="H819" s="2" t="inlineStr">
@@ -37251,7 +37251,7 @@
       </c>
       <c r="G820" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:46.431445+07:00</t>
+          <t>2026-10-30T09:57:26.960653+07:00</t>
         </is>
       </c>
       <c r="H820" s="2" t="inlineStr">
@@ -37292,7 +37292,7 @@
       </c>
       <c r="G821" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.493622+07:00</t>
+          <t>2026-10-30T09:57:23.402806+07:00</t>
         </is>
       </c>
       <c r="H821" s="2" t="inlineStr">
@@ -37333,7 +37333,7 @@
       </c>
       <c r="G822" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.687237+07:00</t>
+          <t>2026-10-30T09:57:37.572573+07:00</t>
         </is>
       </c>
       <c r="H822" s="2" t="inlineStr">
@@ -37374,7 +37374,7 @@
       </c>
       <c r="G823" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:04.579683+07:00</t>
+          <t>2026-10-30T09:57:42.919200+07:00</t>
         </is>
       </c>
       <c r="H823" s="2" t="inlineStr">
@@ -37415,7 +37415,7 @@
       </c>
       <c r="G824" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:25.879945+07:00</t>
+          <t>2026-10-30T09:57:08.215829+07:00</t>
         </is>
       </c>
       <c r="H824" s="2" t="inlineStr">
@@ -37456,7 +37456,7 @@
       </c>
       <c r="G825" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:54.894727+07:00</t>
+          <t>2026-10-30T09:57:34.006892+07:00</t>
         </is>
       </c>
       <c r="H825" s="2" t="inlineStr">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="G826" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.845442+07:00</t>
+          <t>2026-10-30T09:57:10.943711+07:00</t>
         </is>
       </c>
       <c r="H826" s="2" t="inlineStr">
@@ -37538,7 +37538,7 @@
       </c>
       <c r="G827" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.041011+07:00</t>
+          <t>2026-10-30T09:57:32.265183+07:00</t>
         </is>
       </c>
       <c r="H827" s="2" t="inlineStr">
@@ -37579,7 +37579,7 @@
       </c>
       <c r="G828" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:56.702074+07:00</t>
+          <t>2026-10-30T09:57:35.857622+07:00</t>
         </is>
       </c>
       <c r="H828" s="2" t="inlineStr">
@@ -37620,7 +37620,7 @@
       </c>
       <c r="G829" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.951722+07:00</t>
+          <t>2026-10-30T09:57:30.533140+07:00</t>
         </is>
       </c>
       <c r="H829" s="2" t="inlineStr">
@@ -37661,7 +37661,7 @@
       </c>
       <c r="G830" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:53.042937+07:00</t>
+          <t>2026-10-30T09:57:32.317455+07:00</t>
         </is>
       </c>
       <c r="H830" s="2" t="inlineStr">
@@ -37702,7 +37702,7 @@
       </c>
       <c r="G831" t="inlineStr">
         <is>
-          <t>2026-10-30T09:39:00.671439+07:00</t>
+          <t>2026-10-30T09:57:39.416999+07:00</t>
         </is>
       </c>
       <c r="H831" s="2" t="inlineStr">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="G832" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.594388+07:00</t>
+          <t>2026-10-30T09:57:28.723532+07:00</t>
         </is>
       </c>
       <c r="H832" s="2" t="inlineStr">
@@ -37784,7 +37784,7 @@
       </c>
       <c r="G833" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:36.135506+07:00</t>
+          <t>2026-10-30T09:57:18.062473+07:00</t>
         </is>
       </c>
       <c r="H833" s="2" t="inlineStr">
@@ -37825,7 +37825,7 @@
       </c>
       <c r="G834" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.148730+07:00</t>
+          <t>2026-10-30T09:57:21.606230+07:00</t>
         </is>
       </c>
       <c r="H834" s="2" t="inlineStr">
@@ -37866,7 +37866,7 @@
       </c>
       <c r="G835" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:42.492614+07:00</t>
+          <t>2026-10-30T09:57:23.362870+07:00</t>
         </is>
       </c>
       <c r="H835" s="2" t="inlineStr">
@@ -37907,7 +37907,7 @@
       </c>
       <c r="G836" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:44.615639+07:00</t>
+          <t>2026-10-30T09:57:25.199315+07:00</t>
         </is>
       </c>
       <c r="H836" s="2" t="inlineStr">
@@ -37948,7 +37948,7 @@
       </c>
       <c r="G837" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.191795+07:00</t>
+          <t>2026-10-30T09:57:21.654901+07:00</t>
         </is>
       </c>
       <c r="H837" s="2" t="inlineStr">
@@ -37989,7 +37989,7 @@
       </c>
       <c r="G838" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.790040+07:00</t>
+          <t>2026-10-30T09:57:15.526309+07:00</t>
         </is>
       </c>
       <c r="H838" s="2" t="inlineStr">
@@ -38030,7 +38030,7 @@
       </c>
       <c r="G839" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:48.689393+07:00</t>
+          <t>2026-10-30T09:57:28.754114+07:00</t>
         </is>
       </c>
       <c r="H839" s="2" t="inlineStr">
@@ -38071,7 +38071,7 @@
       </c>
       <c r="G840" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:37.816883+07:00</t>
+          <t>2026-10-30T09:57:19.840148+07:00</t>
         </is>
       </c>
       <c r="H840" s="2" t="inlineStr">
@@ -38112,7 +38112,7 @@
       </c>
       <c r="G841" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:50.949592+07:00</t>
+          <t>2026-10-30T09:57:30.484548+07:00</t>
         </is>
       </c>
       <c r="H841" s="2" t="inlineStr">
@@ -38153,7 +38153,7 @@
       </c>
       <c r="G842" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.847007+07:00</t>
+          <t>2026-10-30T09:57:10.944880+07:00</t>
         </is>
       </c>
       <c r="H842" s="2" t="inlineStr">
@@ -38194,7 +38194,7 @@
       </c>
       <c r="G843" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:28.846368+07:00</t>
+          <t>2026-10-30T09:57:10.944223+07:00</t>
         </is>
       </c>
       <c r="H843" s="2" t="inlineStr">
@@ -38235,7 +38235,7 @@
       </c>
       <c r="G844" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:58.905897+07:00</t>
+          <t>2026-10-30T09:57:37.665275+07:00</t>
         </is>
       </c>
       <c r="H844" s="2" t="inlineStr">
@@ -38276,7 +38276,7 @@
       </c>
       <c r="G845" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:37.816068+07:00</t>
+          <t>2026-10-30T09:57:19.827952+07:00</t>
         </is>
       </c>
       <c r="H845" s="2" t="inlineStr">
@@ -38317,7 +38317,7 @@
       </c>
       <c r="G846" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:40.150024+07:00</t>
+          <t>2026-10-30T09:57:21.607153+07:00</t>
         </is>
       </c>
       <c r="H846" s="2" t="inlineStr">
@@ -38358,7 +38358,7 @@
       </c>
       <c r="G847" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:33.788912+07:00</t>
+          <t>2026-10-30T09:57:15.300415+07:00</t>
         </is>
       </c>
       <c r="H847" s="2" t="inlineStr">
@@ -38399,7 +38399,7 @@
       </c>
       <c r="G848" t="inlineStr">
         <is>
-          <t>2026-10-30T09:38:30.915990+07:00</t>
+          <t>2026-10-30T09:57:13.561604+07:00</t>
         </is>
       </c>
       <c r="H848" s="2" t="inlineStr">

</xml_diff>